<commit_message>
docs(configcenter): diversify Go bugfix prompts
</commit_message>
<xml_diff>
--- a/go-config-center-bug-prompts.xlsx
+++ b/go-config-center-bug-prompts.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugfix Prompts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Bugfix Prompts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bugfix Prompts'!$A$1:$D$11</definedName>
@@ -51,13 +51,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -429,27 +432,27 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>task_type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Go Bugfix 提示词</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Bugfix定位提示词</t>
         </is>
@@ -464,10 +467,10 @@
           <t>diagnosis</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>配置中心的事件总线在订阅和发布之间使用了不一致的锁语义，同时发布路径又可能异步执行。请从 `internal/event/hub.go` 的 groups/history 生命周期、`internal/service/releases.go` 的广播调用链入手，构造多个订阅者并连续发布配置版本，判断是锁升级、并发 map 访问、关闭 channel 还是事件丢失导致请求间歇性失败。先别改代码，帮我定位根因</t>
+          <t>配置中心的 SSE Hub 在并发场景下出现很难复现的订阅中断：同一应用环境同时挂着多个客户端，发布线程不断写入事件，客户端又会反复断开重连。请从 internal/event/hub.go 的订阅集合、历史队列和 channel 关闭路径开始，结合 internal/service/releases.go 的广播调用时序，判断问题究竟是锁覆盖不足、关闭后的发送，还是清理流程遗漏导致的，并给出稳定复现所需的竞态顺序。先别改代码，帮我定位根因</t>
         </is>
       </c>
     </row>
@@ -480,10 +483,10 @@
           <t>diagnosis</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>一次发布请求返回成功后，客户端的 SSE 订阅却稳定收不到对应的 config.changed 事件。请沿着 `internal/transport/http/releases.go`、`internal/service/releases.go` 的请求 context 传递，检查 handler 返回时 cancel、广播执行时机和 Hub 发布之间的生命周期关系，说明为什么数据库已经提交但通知链路会静默丢失。先别改代码，帮我定位根因</t>
+          <t>有一类发布请求在接口已经返回 200 后，订阅端却永远等不到 config.changed；如果发布过程中客户端主动断开，问题出现得更频繁。请沿着 internal/transport/http/releases.go 到 internal/service/releases.go 的 context、goroutine 和事件发送链路排查，区分“请求取消被错误传到后台任务”和“通知尚未入队就被提前结束”这两种可能，最后指出具体的生命周期断点。先别改代码，帮我定位根因</t>
         </is>
       </c>
     </row>
@@ -496,10 +499,10 @@
           <t>diagnosis</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>当客户端请求不存在的应用或环境时，服务应返回 NOT_FOUND，但某些路径会被包装成 INTERNAL_ERROR，导致 HTTP 状态和错误码都不对。请追踪 `internal/repository/sqlite_base.go` 的 SQLite 错误映射、`internal/service/applications.go` 的跨层转发以及 `errors.Is/errors.As` 的判定链，定位错误类型在哪一层被破坏。先别改代码，帮我定位根因</t>
+          <t>调用应用、环境或版本查询接口时，底层明明返回了“记录不存在”，HTTP 层却偶尔给出 500，偶尔又返回业务 NOT_FOUND。请追踪 internal/repository/sqlite_base.go 的错误转换、internal/service/applications.go 的再次包装以及 transport 层 errors.Is/errors.As 的判断过程，找出哪一次跨层传递改变了错误身份，并说明为什么结果会随调用路径不同而变化。先别改代码，帮我定位根因</t>
         </is>
       </c>
     </row>
@@ -512,10 +515,10 @@
           <t>diagnosis</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>读取历史发布版本的管理接口在处理正常发布版本时出现运行时崩溃。请从 `internal/transport/http/releases.go` 对 release 元数据的后处理追到 `internal/service/releases.go` 和 `domain.Release` 的 SourceVersion 约定，找出哪个合法状态被错误地当成必有指针，并说明 panic 如何穿过业务层、又如何被 HTTP 恢复中间件改写成统一错误。先别改代码，帮我定位根因</t>
+          <t>管理端打开发布历史时，普通发布记录会触发运行时崩溃，但回滚记录反而正常。请检查 internal/transport/http/releases.go 对 release 元数据的组装、internal/service/releases.go 的返回值以及 domain.Release 中 SourceVersion 的可选语义，定位哪个分支把 nil 当成必有对象使用，并说明 panic 在恢复中间件之后为何只剩下统一的内部错误。先别改代码，帮我定位根因</t>
         </is>
       </c>
     </row>
@@ -530,10 +533,10 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>修复配置中心发布后的 SSE 通知并发缺陷：当多个客户端订阅同一应用环境、发布请求连续到达时，`internal/event/hub.go` 的订阅表、历史缓存和 channel 关闭必须保持一致，不能出现 concurrent map 访问、向已关闭 channel 写入、重复关闭或订阅者永久泄漏。请保留 Last-Event-ID 重放语义，并让 `internal/service/releases.go` 的通知调用在高并发下稳定工作。</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
+          <t>并发压测发布与订阅流程时，internal/event/hub.go 需要同时维护订阅者、历史事件和退出通知。请修正这条链路，使客户端断开、Hub 关闭、事件广播交错发生时都不会向已关闭 channel 写入、重复 close 或遗留 goroutine；多个订阅者仍要按 Last-Event-ID 获得正确的重放结果，internal/service/releases.go 的发布接口也不能因单个慢客户端卡住。</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n"/>
     </row>
     <row r="7" ht="92" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -546,10 +549,10 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>修复发布请求的 context 生命周期问题：HTTP handler 返回后不应让已经成功提交的发布丢失通知，也不能为了保活而把请求取消语义彻底切断。请调整 `internal/transport/http/releases.go` 与 `internal/service/releases.go` 的 context 传递和广播时序，使数据库提交、事件发布和客户端取消之间的边界明确，并验证客户端能稳定收到 config.changed。</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
+          <t>发布落库成功后，通知任务必须拥有独立且可控的生命周期：HTTP 请求结束不应把已经提交的变更静默取消，但调用方真正取消时又不能继续无限运行。请调整 internal/transport/http/releases.go 与 internal/service/releases.go 的 context 派生、取消和异步广播边界，处理超时与客户端断连两条路径，并用连续发布验证每个订阅端都能收到对应版本事件。</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n"/>
     </row>
     <row r="8" ht="92" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -562,10 +565,10 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>修复错误传播链路：SQLite 查询找不到应用、环境或版本时，外层必须仍能通过 `errors.Is/errors.As` 识别领域错误并返回正确的 NOT_FOUND 或其他业务码。请检查 `internal/repository/sqlite_base.go`、`internal/service/applications.go` 与 HTTP 错误映射之间的包装方式，避免用字符串拼接丢失 Cause，也不要把所有底层错误粗暴改成同一个状态。</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
+          <t>请修复“资源不存在”在 repository、service、HTTP 三层之间传播时丢失类型信息的问题。重点处理 internal/repository/sqlite_base.go 的 SQLite 错误映射和 internal/service/applications.go 的包装方式，让 errors.Is/errors.As 在最外层仍可识别领域错误；不同错误应分别映射到 NOT_FOUND、冲突或 INTERNAL_ERROR，不能再依赖错误字符串或把底层 Cause 藏掉。</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n"/>
     </row>
     <row r="9" ht="92" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -578,10 +581,10 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>修复历史发布版本读取时的 nil 指针崩溃。普通 publish 版本没有 SourceVersion，rollback 版本才有来源版本；请在 `internal/service/releases.go` 和 `internal/transport/http/releases.go` 之间建立正确的可选字段处理，保证管理接口既能返回普通发布，也能返回回滚元数据，且 panic 恢复中间件不再掩盖真实业务结果。</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
+          <t>历史版本接口对 release.SourceVersion 的处理需要区分普通 publish 和 rollback：前者没有来源版本并不代表数据损坏。请在 internal/service/releases.go 和 internal/transport/http/releases.go 中补齐可选字段的分支处理，消除合法请求的 nil 解引用，同时保持回滚记录的来源版本、发布时间和配置内容都能正常返回。</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n"/>
     </row>
     <row r="10" ht="92" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -594,10 +597,10 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>修复 SSE 历史重放造成的状态污染：`internal/event/hub.go` 的 replay 筛选不能复用 history 的底层数组，否则新订阅重放时会覆盖全局事件缓存；`internal/transport/http/subscription.go` 也不能把没有 Last-Event-ID 的首次连接强行当成断线重连。请保持首次连接只发送 ready、断线按 Last-Event-ID 精确重放，并验证多次订阅后历史事件顺序和后续发布通知都不被破坏。</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
+          <t>新客户端首次建立 SSE 连接时只应收到 ready，带有 Last-Event-ID 的重连才需要筛选历史记录。请修复 internal/event/hub.go 的历史重放实现，避免用共享底层数组做筛选导致全局 history 被改写，也要让多次重连不会重复或跳过事件；验证一个客户端的重放操作不会改变其他客户端随后看到的顺序。</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n"/>
     </row>
     <row r="11" ht="92" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -610,10 +613,10 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>修复草稿写入路径中的资源生命周期问题。当前 `internal/repository/sqlite_configs.go` 在批量插入 draft_items 时可能把 defer 放在循环里，长批量请求会积累大量 statement/连接资源；同时检查 `internal/service/configurations.go` 的输入副本和事务失败回滚，确保高频保存不会耗尽 SQLite 资源、残留半写入状态或污染下一次请求。</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
+          <t>批量保存配置草稿时，internal/repository/sqlite_configs.go 不能把每轮 Prepare/Query 的 defer 累积到整个请求结束；在较大的 item 列表上这会拖住 SQLite 资源，并让失败事务留下可见的半成品。请重新安排 statement、rows 和事务的释放时机，检查 internal/service/configurations.go 的输入副本与回滚路径，确保连续保存不会耗尽资源或污染下一次请求。</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D11"/>

</xml_diff>